<commit_message>
feat(tesis): aplica cambios de metodologia, datos y graficos y reestima el modelo
- Binarias presidenciales por mandato (Wald/LR) y variante sin ellas; Cholesky en dos ordenes.
- Cuatro transiciones de la tasa de la FED; muestra consolidada desde 2002; quiebres recalculados.
- 1.000 replicas; regla de reserva de rezagos; apertura de la varianza externa (VIX, FED, costo directo).
- Resultados reestimados: H1a y H1b se mantienen; H2 queda parcialmente respaldada.
- Texto, apendice, figuras, hoja de numeros y guia de ejecucion actualizados; PDF regenerado.
</commit_message>
<xml_diff>
--- a/tesis_oficial_borradores/para_el_grupo/Datos_y_resultados.xlsx
+++ b/tesis_oficial_borradores/para_el_grupo/Datos_y_resultados.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1963" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1969" uniqueCount="411">
   <si>
     <t>Hoja</t>
   </si>
@@ -78,7 +78,7 @@
     <t>Estilo_FMI</t>
   </si>
   <si>
-    <t>Base trimestral 1996-2025: EMBI+, TCRM, PIB real y demas variables</t>
+    <t>Base trimestral 1996-2025: EMBI, TCRM, PIB real y demas variables</t>
   </si>
   <si>
     <t>Deuda en % del PIB: bruta_federal_pib (principal) y deuda_consolidada_neta_nominal_pib (extension)</t>
@@ -1192,6 +1192,15 @@
   </si>
   <si>
     <t>vshare_externo</t>
+  </si>
+  <si>
+    <t>vshare_externo_vix</t>
+  </si>
+  <si>
+    <t>vshare_externo_fed</t>
+  </si>
+  <si>
+    <t>vshare_externo_fed_directo</t>
   </si>
   <si>
     <t>var_total_2035</t>
@@ -1738,16 +1747,16 @@
         <v>32</v>
       </c>
       <c r="B2">
-        <v>1.427249030783867</v>
+        <v>1.316436120538078</v>
       </c>
       <c r="C2">
-        <v>0.7117144562759263</v>
+        <v>0.6770611456348301</v>
       </c>
       <c r="D2">
-        <v>-1.110223024625156E-16</v>
+        <v>-1.470014339310516E-16</v>
       </c>
       <c r="E2">
-        <v>-3.33066907387547E-16</v>
+        <v>-8.686317283924251E-17</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1755,16 +1764,16 @@
         <v>361</v>
       </c>
       <c r="B3">
-        <v>-0.3261230969812968</v>
+        <v>-0.2771633073781988</v>
       </c>
       <c r="C3">
-        <v>2.846857825103705</v>
+        <v>2.708244582539319</v>
       </c>
       <c r="D3">
-        <v>-8.881784197001252E-16</v>
+        <v>-7.634094047526119E-17</v>
       </c>
       <c r="E3">
-        <v>-1.554312234475219E-15</v>
+        <v>-1.039783816359058E-15</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1772,16 +1781,16 @@
         <v>35</v>
       </c>
       <c r="B4">
-        <v>-116.7523293103676</v>
+        <v>-85.3604981125191</v>
       </c>
       <c r="C4">
-        <v>-47.88998550596051</v>
+        <v>-22.50356700746238</v>
       </c>
       <c r="D4">
-        <v>461.4094735754815</v>
+        <v>376.4842162951616</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2.550161905246084E-14</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1789,16 +1798,16 @@
         <v>34</v>
       </c>
       <c r="B5">
-        <v>0.0209398383832931</v>
+        <v>0.013561049148703</v>
       </c>
       <c r="C5">
-        <v>-0.010853998773901</v>
+        <v>-0.0075208656961326</v>
       </c>
       <c r="D5">
-        <v>0.0114062133199225</v>
+        <v>-0.0022727642449182</v>
       </c>
       <c r="E5">
-        <v>0.1016655773985354</v>
+        <v>0.1058686921373418</v>
       </c>
     </row>
   </sheetData>
@@ -1808,7 +1817,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1830,13 +1839,13 @@
         <v>363</v>
       </c>
       <c r="B2">
-        <v>0.3177</v>
+        <v>0.27685</v>
       </c>
       <c r="C2">
-        <v>0.2523499999999999</v>
+        <v>0.2056</v>
       </c>
       <c r="D2">
-        <v>0.3644499999999999</v>
+        <v>0.34675</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1844,13 +1853,13 @@
         <v>364</v>
       </c>
       <c r="B3">
-        <v>0.31015</v>
+        <v>0.2901</v>
       </c>
       <c r="C3">
-        <v>0.26825</v>
+        <v>0.2502</v>
       </c>
       <c r="D3">
-        <v>0.3563499999999999</v>
+        <v>0.3612000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1858,13 +1867,13 @@
         <v>365</v>
       </c>
       <c r="B4">
-        <v>45.31661790352911</v>
+        <v>45.01178004002475</v>
       </c>
       <c r="C4">
-        <v>43.37424529692515</v>
+        <v>40.70988769573533</v>
       </c>
       <c r="D4">
-        <v>53.29212207649692</v>
+        <v>50.9504605943194</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1872,13 +1881,13 @@
         <v>366</v>
       </c>
       <c r="B5">
-        <v>0.3254</v>
+        <v>0.2868</v>
       </c>
       <c r="C5">
-        <v>0.2638</v>
+        <v>0.2106</v>
       </c>
       <c r="D5">
-        <v>0.37285</v>
+        <v>0.3576</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1886,13 +1895,13 @@
         <v>367</v>
       </c>
       <c r="B6">
-        <v>0.32105</v>
+        <v>0.3089</v>
       </c>
       <c r="C6">
-        <v>0.2841</v>
+        <v>0.2637500000000001</v>
       </c>
       <c r="D6">
-        <v>0.37115</v>
+        <v>0.3838</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1900,13 +1909,13 @@
         <v>368</v>
       </c>
       <c r="B7">
-        <v>46.33401816938314</v>
+        <v>46.99962638308448</v>
       </c>
       <c r="C7">
-        <v>43.91023684203677</v>
+        <v>41.62925328452584</v>
       </c>
       <c r="D7">
-        <v>54.7532938550486</v>
+        <v>53.61703629162203</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1914,13 +1923,13 @@
         <v>369</v>
       </c>
       <c r="B8">
-        <v>0.3679</v>
+        <v>0.34385</v>
       </c>
       <c r="C8">
-        <v>0.2788</v>
+        <v>0.2687</v>
       </c>
       <c r="D8">
-        <v>0.428</v>
+        <v>0.4297499999999999</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1928,13 +1937,13 @@
         <v>370</v>
       </c>
       <c r="B9">
-        <v>0.40695</v>
+        <v>0.47395</v>
       </c>
       <c r="C9">
-        <v>0.3476</v>
+        <v>0.35185</v>
       </c>
       <c r="D9">
-        <v>0.4889999999999999</v>
+        <v>0.6138999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1942,13 +1951,13 @@
         <v>371</v>
       </c>
       <c r="B10">
-        <v>54.32281591727576</v>
+        <v>64.30082211773031</v>
       </c>
       <c r="C10">
-        <v>44.63322675541914</v>
+        <v>41.95851642657208</v>
       </c>
       <c r="D10">
-        <v>66.09462959717717</v>
+        <v>79.70936171707935</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1956,13 +1965,13 @@
         <v>372</v>
       </c>
       <c r="B11">
-        <v>0.3561</v>
+        <v>0.29655</v>
       </c>
       <c r="C11">
-        <v>0.3091</v>
+        <v>0.2350999999999999</v>
       </c>
       <c r="D11">
-        <v>0.4113</v>
+        <v>0.3731</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1970,13 +1979,13 @@
         <v>373</v>
       </c>
       <c r="B12">
-        <v>0.25795</v>
+        <v>0.2004</v>
       </c>
       <c r="C12">
-        <v>0.21785</v>
+        <v>0.1727999999999999</v>
       </c>
       <c r="D12">
-        <v>0.3119</v>
+        <v>0.2668</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1984,13 +1993,13 @@
         <v>374</v>
       </c>
       <c r="B13">
-        <v>0.35565</v>
+        <v>0.3027</v>
       </c>
       <c r="C13">
-        <v>0.31225</v>
+        <v>0.2604000000000001</v>
       </c>
       <c r="D13">
-        <v>0.4193</v>
+        <v>0.3734</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1998,13 +2007,13 @@
         <v>375</v>
       </c>
       <c r="B14">
-        <v>0.2932</v>
+        <v>0.2515</v>
       </c>
       <c r="C14">
-        <v>0.2504</v>
+        <v>0.199</v>
       </c>
       <c r="D14">
-        <v>0.3655</v>
+        <v>0.347</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2012,13 +2021,13 @@
         <v>376</v>
       </c>
       <c r="B15">
-        <v>46.63948146093939</v>
+        <v>40.48473036617251</v>
       </c>
       <c r="C15">
-        <v>36.79910302584346</v>
+        <v>32.36757292839395</v>
       </c>
       <c r="D15">
-        <v>60.95786313310419</v>
+        <v>54.49125681057952</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2026,13 +2035,13 @@
         <v>377</v>
       </c>
       <c r="B16">
-        <v>53.05987110964295</v>
+        <v>52.88758425028549</v>
       </c>
       <c r="C16">
-        <v>52.23012611833906</v>
+        <v>51.83988946986869</v>
       </c>
       <c r="D16">
-        <v>56.82432654854698</v>
+        <v>55.19878815825226</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2040,13 +2049,13 @@
         <v>378</v>
       </c>
       <c r="B17">
-        <v>0.0077</v>
+        <v>0.009950000000000001</v>
       </c>
       <c r="C17">
-        <v>0.0014</v>
+        <v>-0.0030999999999999</v>
       </c>
       <c r="D17">
-        <v>0.01445</v>
+        <v>0.0159</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2054,13 +2063,13 @@
         <v>379</v>
       </c>
       <c r="B18">
-        <v>0.0109</v>
+        <v>0.0187999999999999</v>
       </c>
       <c r="C18">
-        <v>0.00175</v>
+        <v>0.0025999999999999</v>
       </c>
       <c r="D18">
-        <v>0.0188</v>
+        <v>0.0315999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2068,13 +2077,13 @@
         <v>380</v>
       </c>
       <c r="B19">
-        <v>1.017400265854029</v>
+        <v>1.987846343059722</v>
       </c>
       <c r="C19">
-        <v>0.0175368047116322</v>
+        <v>0.3565840799157938</v>
       </c>
       <c r="D19">
-        <v>1.833363049707731</v>
+        <v>3.216609740853269</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2082,13 +2091,13 @@
         <v>381</v>
       </c>
       <c r="B20">
-        <v>0.0502</v>
+        <v>0.067</v>
       </c>
       <c r="C20">
-        <v>0.0023</v>
+        <v>0.00595</v>
       </c>
       <c r="D20">
-        <v>0.0915</v>
+        <v>0.12805</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2096,13 +2105,13 @@
         <v>382</v>
       </c>
       <c r="B21">
-        <v>0.0968</v>
+        <v>0.1838499999999999</v>
       </c>
       <c r="C21">
-        <v>0.0415</v>
+        <v>0.06265</v>
       </c>
       <c r="D21">
-        <v>0.1597</v>
+        <v>0.2906999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2110,13 +2119,13 @@
         <v>383</v>
       </c>
       <c r="B22">
-        <v>9.006198013746655</v>
+        <v>19.28904207770555</v>
       </c>
       <c r="C22">
-        <v>0.2726336127508659</v>
+        <v>-0.3148925418898756</v>
       </c>
       <c r="D22">
-        <v>16.2291407968505</v>
+        <v>31.34279913377381</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2124,13 +2133,13 @@
         <v>384</v>
       </c>
       <c r="B23">
-        <v>10.82711452920347</v>
+        <v>1.579038188322416</v>
       </c>
       <c r="C23">
-        <v>6.061089373416742</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>21.33980290026658</v>
+        <v>3.067315506632514</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2138,13 +2147,13 @@
         <v>385</v>
       </c>
       <c r="B24">
-        <v>11.99121510040592</v>
+        <v>10.70677095939053</v>
       </c>
       <c r="C24">
-        <v>0.1867983596923466</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>21.23984856449255</v>
+        <v>19.79783478607243</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2152,13 +2161,13 @@
         <v>386</v>
       </c>
       <c r="B25">
-        <v>32.25674465156604</v>
+        <v>28.31047102047497</v>
       </c>
       <c r="C25">
-        <v>16.76057727853612</v>
+        <v>14.04127823130952</v>
       </c>
       <c r="D25">
-        <v>48.92062770644062</v>
+        <v>48.81617132268431</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2166,13 +2175,13 @@
         <v>387</v>
       </c>
       <c r="B26">
-        <v>44.92492571882459</v>
+        <v>59.40371983181209</v>
       </c>
       <c r="C26">
-        <v>14.63295890389313</v>
+        <v>30.45889528603178</v>
       </c>
       <c r="D26">
-        <v>58.98496648246164</v>
+        <v>78.53262942842997</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2180,13 +2189,13 @@
         <v>388</v>
       </c>
       <c r="B27">
-        <v>474.740687411821</v>
+        <v>113.2287725945662</v>
       </c>
       <c r="C27">
-        <v>-166.9458227993516</v>
+        <v>3.955298664255338</v>
       </c>
       <c r="D27">
-        <v>833.5341753660967</v>
+        <v>174.8770986579737</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2194,13 +2203,13 @@
         <v>389</v>
       </c>
       <c r="B28">
-        <v>651.4906983919047</v>
+        <v>13.28076355403068</v>
       </c>
       <c r="C28">
-        <v>-643.3071129175351</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>1160.005633019593</v>
+        <v>23.62694963042727</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2208,13 +2217,13 @@
         <v>390</v>
       </c>
       <c r="B29">
-        <v>78.34577094159306</v>
+        <v>7.564345540939048</v>
       </c>
       <c r="C29">
-        <v>57.32039419946685</v>
+        <v>0</v>
       </c>
       <c r="D29">
-        <v>87.87782125316659</v>
+        <v>11.44543899042563</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2222,7 +2231,13 @@
         <v>391</v>
       </c>
       <c r="B30">
-        <v>8.602527573332637</v>
+        <v>441.0130967801855</v>
+      </c>
+      <c r="C30">
+        <v>-267.640261492618</v>
+      </c>
+      <c r="D30">
+        <v>769.797160971215</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2230,7 +2245,13 @@
         <v>392</v>
       </c>
       <c r="B31">
-        <v>53.90665208438045</v>
+        <v>606.1012390752727</v>
+      </c>
+      <c r="C31">
+        <v>-496.7967273356105</v>
+      </c>
+      <c r="D31">
+        <v>1086.811122467577</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2238,7 +2259,13 @@
         <v>393</v>
       </c>
       <c r="B32">
-        <v>42.74134704670094</v>
+        <v>96.84192362335516</v>
+      </c>
+      <c r="C32">
+        <v>93.86536898673498</v>
+      </c>
+      <c r="D32">
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -2246,7 +2273,7 @@
         <v>394</v>
       </c>
       <c r="B33">
-        <v>0.0032921627389908</v>
+        <v>14.80361697387622</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -2254,7 +2281,31 @@
         <v>395</v>
       </c>
       <c r="B34">
-        <v>0.003270756621181</v>
+        <v>53.90665208438045</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>396</v>
+      </c>
+      <c r="B35">
+        <v>42.74134704670094</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>397</v>
+      </c>
+      <c r="B36">
+        <v>0.0031638906231094</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>398</v>
+      </c>
+      <c r="B37">
+        <v>0.0032089093941711</v>
       </c>
     </row>
   </sheetData>
@@ -2272,22 +2323,22 @@
         <v>220</v>
       </c>
       <c r="B1" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="C1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="D1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E1" t="s">
         <v>265</v>
       </c>
       <c r="F1" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="G1" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="H1" t="s">
         <v>266</v>
@@ -2324,25 +2375,25 @@
         <v>2026</v>
       </c>
       <c r="B3">
-        <v>65.85137652477287</v>
+        <v>67.22560373253812</v>
       </c>
       <c r="C3">
-        <v>67.16633785043216</v>
+        <v>67.85652870018815</v>
       </c>
       <c r="D3">
-        <v>69.1799701416051</v>
+        <v>70.26062091071461</v>
       </c>
       <c r="E3">
-        <v>72.83253632478176</v>
+        <v>72.49012585222668</v>
       </c>
       <c r="F3">
-        <v>75.84424564042864</v>
+        <v>74.94844870587002</v>
       </c>
       <c r="G3">
-        <v>84.92079834738904</v>
+        <v>80.40906681407122</v>
       </c>
       <c r="H3">
-        <v>90.19593094698909</v>
+        <v>87.65189295990012</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2350,25 +2401,25 @@
         <v>2027</v>
       </c>
       <c r="B4">
-        <v>56.13436291116239</v>
+        <v>59.41096470980451</v>
       </c>
       <c r="C4">
-        <v>61.80594768779546</v>
+        <v>64.03676038117575</v>
       </c>
       <c r="D4">
-        <v>65.03188227971397</v>
+        <v>65.79350094966532</v>
       </c>
       <c r="E4">
-        <v>70.04484505705689</v>
+        <v>69.16224928955232</v>
       </c>
       <c r="F4">
-        <v>75.07127537510601</v>
+        <v>73.06896771105657</v>
       </c>
       <c r="G4">
-        <v>84.15211143739454</v>
+        <v>85.55269247215374</v>
       </c>
       <c r="H4">
-        <v>89.42688670242553</v>
+        <v>88.93537268861277</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2376,25 +2427,25 @@
         <v>2028</v>
       </c>
       <c r="B5">
-        <v>52.03865539417852</v>
+        <v>54.13746716150237</v>
       </c>
       <c r="C5">
-        <v>55.26318425170105</v>
+        <v>56.74596443860114</v>
       </c>
       <c r="D5">
-        <v>59.99141579401542</v>
+        <v>60.43079470190232</v>
       </c>
       <c r="E5">
-        <v>64.95607146371236</v>
+        <v>64.78784092752194</v>
       </c>
       <c r="F5">
-        <v>70.49129910098634</v>
+        <v>70.22735798983018</v>
       </c>
       <c r="G5">
-        <v>78.23466709781502</v>
+        <v>75.91066969894717</v>
       </c>
       <c r="H5">
-        <v>83.08485990049299</v>
+        <v>80.432426052011</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2402,25 +2453,25 @@
         <v>2029</v>
       </c>
       <c r="B6">
-        <v>44.06003872187772</v>
+        <v>46.69308208091125</v>
       </c>
       <c r="C6">
-        <v>47.34721155695779</v>
+        <v>50.1864692173877</v>
       </c>
       <c r="D6">
-        <v>53.76141808603769</v>
+        <v>54.43626598641902</v>
       </c>
       <c r="E6">
-        <v>60.38003799404573</v>
+        <v>60.14461389538531</v>
       </c>
       <c r="F6">
-        <v>67.97327275562087</v>
+        <v>66.81833797785434</v>
       </c>
       <c r="G6">
-        <v>77.08519321970047</v>
+        <v>75.22388552804902</v>
       </c>
       <c r="H6">
-        <v>82.06798484033685</v>
+        <v>80.3795175623616</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2428,25 +2479,25 @@
         <v>2030</v>
       </c>
       <c r="B7">
-        <v>39.35095582842837</v>
+        <v>41.89189337117663</v>
       </c>
       <c r="C7">
-        <v>43.11170497329176</v>
+        <v>45.40677969478156</v>
       </c>
       <c r="D7">
-        <v>49.82173686766699</v>
+        <v>50.45234720922301</v>
       </c>
       <c r="E7">
-        <v>56.99878243964051</v>
+        <v>56.84343969488502</v>
       </c>
       <c r="F7">
-        <v>65.12127871268423</v>
+        <v>64.14382917659289</v>
       </c>
       <c r="G7">
-        <v>73.58841714313306</v>
+        <v>71.58595091587925</v>
       </c>
       <c r="H7">
-        <v>79.42300275750632</v>
+        <v>76.41593012527468</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2454,25 +2505,25 @@
         <v>2031</v>
       </c>
       <c r="B8">
-        <v>33.15961675573696</v>
+        <v>35.96885343217358</v>
       </c>
       <c r="C8">
-        <v>37.12422626438015</v>
+        <v>39.79789089600312</v>
       </c>
       <c r="D8">
-        <v>44.4871804312068</v>
+        <v>45.70520337164501</v>
       </c>
       <c r="E8">
-        <v>53.05987110964295</v>
+        <v>52.88758425028549</v>
       </c>
       <c r="F8">
-        <v>62.66030023857462</v>
+        <v>61.37307834043703</v>
       </c>
       <c r="G8">
-        <v>73.07068096449436</v>
+        <v>70.48104002735245</v>
       </c>
       <c r="H8">
-        <v>79.79909821667634</v>
+        <v>76.45358379834609</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2480,25 +2531,25 @@
         <v>2032</v>
       </c>
       <c r="B9">
-        <v>29.1224942046643</v>
+        <v>31.63129543827842</v>
       </c>
       <c r="C9">
-        <v>33.38519755126548</v>
+        <v>35.73517946867621</v>
       </c>
       <c r="D9">
-        <v>41.19154664292238</v>
+        <v>42.27665055560159</v>
       </c>
       <c r="E9">
-        <v>50.81493426626104</v>
+        <v>50.38602925279378</v>
       </c>
       <c r="F9">
-        <v>61.60207166380855</v>
+        <v>59.97773560237039</v>
       </c>
       <c r="G9">
-        <v>72.74604214597491</v>
+        <v>69.9197513183522</v>
       </c>
       <c r="H9">
-        <v>80.47999826379387</v>
+        <v>76.80521690552781</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2506,25 +2557,25 @@
         <v>2033</v>
       </c>
       <c r="B10">
-        <v>23.96413026071417</v>
+        <v>26.73422192899125</v>
       </c>
       <c r="C10">
-        <v>28.64621211742483</v>
+        <v>30.96692174555472</v>
       </c>
       <c r="D10">
-        <v>37.20483725842348</v>
+        <v>38.08443330357645</v>
       </c>
       <c r="E10">
-        <v>48.02782092907886</v>
+        <v>47.43777434981018</v>
       </c>
       <c r="F10">
-        <v>59.9493141184928</v>
+        <v>58.574628406001</v>
       </c>
       <c r="G10">
-        <v>72.84568771741152</v>
+        <v>70.54134674369418</v>
       </c>
       <c r="H10">
-        <v>81.75487760188348</v>
+        <v>78.90714191016278</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2532,25 +2583,25 @@
         <v>2034</v>
       </c>
       <c r="B11">
-        <v>20.25244726238758</v>
+        <v>22.23743327900901</v>
       </c>
       <c r="C11">
-        <v>24.91183776285942</v>
+        <v>26.77518519931144</v>
       </c>
       <c r="D11">
-        <v>33.95452802800498</v>
+        <v>34.58853515340078</v>
       </c>
       <c r="E11">
-        <v>45.39127710733136</v>
+        <v>44.74974163469347</v>
       </c>
       <c r="F11">
-        <v>58.69396869233008</v>
+        <v>57.11227962209101</v>
       </c>
       <c r="G11">
-        <v>72.97360467818308</v>
+        <v>70.7544314667465</v>
       </c>
       <c r="H11">
-        <v>83.35404540929629</v>
+        <v>80.69264495145603</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2558,25 +2609,25 @@
         <v>2035</v>
       </c>
       <c r="B12">
-        <v>15.8777571988403</v>
+        <v>17.70745442047006</v>
       </c>
       <c r="C12">
-        <v>20.65962813594029</v>
+        <v>22.29283377425641</v>
       </c>
       <c r="D12">
-        <v>30.04622029061395</v>
+        <v>30.37622736775862</v>
       </c>
       <c r="E12">
-        <v>42.08193581906896</v>
+        <v>41.40409041725481</v>
       </c>
       <c r="F12">
-        <v>57.27806922687291</v>
+        <v>55.91698426013981</v>
       </c>
       <c r="G12">
-        <v>73.46343973170632</v>
+        <v>72.32553572199798</v>
       </c>
       <c r="H12">
-        <v>85.47194337063053</v>
+        <v>84.28444331949483</v>
       </c>
     </row>
   </sheetData>
@@ -2591,19 +2642,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B1" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C1" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="D1" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2617,10 +2668,10 @@
         <v>2.299999999999997</v>
       </c>
       <c r="D2">
-        <v>0.3177</v>
+        <v>0.27685</v>
       </c>
       <c r="E2">
-        <v>0.31015</v>
+        <v>0.2901</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2634,10 +2685,10 @@
         <v>2.549999999999997</v>
       </c>
       <c r="D3">
-        <v>0.3022</v>
+        <v>0.26425</v>
       </c>
       <c r="E3">
-        <v>0.29255</v>
+        <v>0.27105</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2651,10 +2702,10 @@
         <v>2.799999999999997</v>
       </c>
       <c r="D4">
-        <v>0.28865</v>
+        <v>0.252</v>
       </c>
       <c r="E4">
-        <v>0.27355</v>
+        <v>0.2518</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2668,10 +2719,10 @@
         <v>3.049999999999997</v>
       </c>
       <c r="D5">
-        <v>0.2751</v>
+        <v>0.2405</v>
       </c>
       <c r="E5">
-        <v>0.2548</v>
+        <v>0.234</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2685,10 +2736,10 @@
         <v>3.299999999999997</v>
       </c>
       <c r="D6">
-        <v>0.2603</v>
+        <v>0.22945</v>
       </c>
       <c r="E6">
-        <v>0.234</v>
+        <v>0.21415</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2702,10 +2753,10 @@
         <v>3.549999999999997</v>
       </c>
       <c r="D7">
-        <v>0.24625</v>
+        <v>0.21715</v>
       </c>
       <c r="E7">
-        <v>0.2157</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2719,10 +2770,10 @@
         <v>3.799999999999997</v>
       </c>
       <c r="D8">
-        <v>0.23225</v>
+        <v>0.2048</v>
       </c>
       <c r="E8">
-        <v>0.19655</v>
+        <v>0.17635</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2736,10 +2787,10 @@
         <v>4.049999999999997</v>
       </c>
       <c r="D9">
-        <v>0.21795</v>
+        <v>0.1936</v>
       </c>
       <c r="E9">
-        <v>0.1784</v>
+        <v>0.1577</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2753,10 +2804,10 @@
         <v>4.299999999999997</v>
       </c>
       <c r="D10">
-        <v>0.2033</v>
+        <v>0.182</v>
       </c>
       <c r="E10">
-        <v>0.15845</v>
+        <v>0.1392</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2770,10 +2821,10 @@
         <v>4.549999999999997</v>
       </c>
       <c r="D11">
-        <v>0.19075</v>
+        <v>0.17105</v>
       </c>
       <c r="E11">
-        <v>0.13955</v>
+        <v>0.1201</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2787,10 +2838,10 @@
         <v>4.799999999999997</v>
       </c>
       <c r="D12">
-        <v>0.17905</v>
+        <v>0.1602</v>
       </c>
       <c r="E12">
-        <v>0.1237</v>
+        <v>0.1021</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2804,10 +2855,10 @@
         <v>5.049999999999997</v>
       </c>
       <c r="D13">
-        <v>0.16575</v>
+        <v>0.14775</v>
       </c>
       <c r="E13">
-        <v>0.1096</v>
+        <v>0.0859</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2821,10 +2872,10 @@
         <v>5.299999999999997</v>
       </c>
       <c r="D14">
-        <v>0.15275</v>
+        <v>0.1364</v>
       </c>
       <c r="E14">
-        <v>0.094</v>
+        <v>0.07105</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2838,10 +2889,10 @@
         <v>5.549999999999997</v>
       </c>
       <c r="D15">
-        <v>0.1401</v>
+        <v>0.1248</v>
       </c>
       <c r="E15">
-        <v>0.08035</v>
+        <v>0.05695</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2855,10 +2906,10 @@
         <v>5.799999999999997</v>
       </c>
       <c r="D16">
-        <v>0.12925</v>
+        <v>0.1138</v>
       </c>
       <c r="E16">
-        <v>0.06725</v>
+        <v>0.04675</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2872,10 +2923,10 @@
         <v>6.049999999999997</v>
       </c>
       <c r="D17">
-        <v>0.1171</v>
+        <v>0.10465</v>
       </c>
       <c r="E17">
-        <v>0.05615</v>
+        <v>0.03765</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2889,10 +2940,10 @@
         <v>6.299999999999997</v>
       </c>
       <c r="D18">
-        <v>0.1078</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="E18">
-        <v>0.0464</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2906,10 +2957,10 @@
         <v>6.549999999999997</v>
       </c>
       <c r="D19">
-        <v>0.09815</v>
+        <v>0.0864</v>
       </c>
       <c r="E19">
-        <v>0.03735</v>
+        <v>0.02115</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2923,10 +2974,10 @@
         <v>6.799999999999997</v>
       </c>
       <c r="D20">
-        <v>0.0888</v>
+        <v>0.07665</v>
       </c>
       <c r="E20">
-        <v>0.03055</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2940,10 +2991,10 @@
         <v>7.049999999999997</v>
       </c>
       <c r="D21">
-        <v>0.07875</v>
+        <v>0.0668</v>
       </c>
       <c r="E21">
-        <v>0.02425</v>
+        <v>0.01155</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2957,10 +3008,10 @@
         <v>7.299999999999997</v>
       </c>
       <c r="D22">
-        <v>0.06950000000000001</v>
+        <v>0.05765</v>
       </c>
       <c r="E22">
-        <v>0.0195</v>
+        <v>0.008200000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2974,10 +3025,10 @@
         <v>7.549999999999997</v>
       </c>
       <c r="D23">
-        <v>0.06225</v>
+        <v>0.0485</v>
       </c>
       <c r="E23">
-        <v>0.0152</v>
+        <v>0.0057</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2991,10 +3042,10 @@
         <v>7.799999999999997</v>
       </c>
       <c r="D24">
-        <v>0.0535</v>
+        <v>0.04075</v>
       </c>
       <c r="E24">
-        <v>0.01255</v>
+        <v>0.00405</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3008,10 +3059,10 @@
         <v>8.049999999999997</v>
       </c>
       <c r="D25">
-        <v>0.0465</v>
+        <v>0.0345</v>
       </c>
       <c r="E25">
-        <v>0.0098</v>
+        <v>0.00255</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3025,10 +3076,10 @@
         <v>8.299999999999997</v>
       </c>
       <c r="D26">
-        <v>0.04055</v>
+        <v>0.02775</v>
       </c>
       <c r="E26">
-        <v>0.0076</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -3042,10 +3093,10 @@
         <v>8.549999999999997</v>
       </c>
       <c r="D27">
-        <v>0.03485</v>
+        <v>0.023</v>
       </c>
       <c r="E27">
-        <v>0.00715</v>
+        <v>0.00125</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3059,10 +3110,10 @@
         <v>8.799999999999997</v>
       </c>
       <c r="D28">
-        <v>0.0294</v>
+        <v>0.01885</v>
       </c>
       <c r="E28">
-        <v>0.0071</v>
+        <v>0.0013</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -3076,10 +3127,10 @@
         <v>9.049999999999995</v>
       </c>
       <c r="D29">
-        <v>0.02425</v>
+        <v>0.0146</v>
       </c>
       <c r="E29">
-        <v>0.00765</v>
+        <v>0.00155</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -3093,10 +3144,10 @@
         <v>9.299999999999995</v>
       </c>
       <c r="D30">
-        <v>0.0198</v>
+        <v>0.0102</v>
       </c>
       <c r="E30">
-        <v>0.007900000000000001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -3110,10 +3161,10 @@
         <v>9.549999999999995</v>
       </c>
       <c r="D31">
-        <v>0.01615</v>
+        <v>0.0076</v>
       </c>
       <c r="E31">
-        <v>0.008999999999999999</v>
+        <v>0.00245</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -3127,10 +3178,10 @@
         <v>9.799999999999995</v>
       </c>
       <c r="D32">
-        <v>0.01365</v>
+        <v>0.00565</v>
       </c>
       <c r="E32">
-        <v>0.01045</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -3144,10 +3195,10 @@
         <v>10.05</v>
       </c>
       <c r="D33">
-        <v>0.0108</v>
+        <v>0.00405</v>
       </c>
       <c r="E33">
-        <v>0.012</v>
+        <v>0.0041</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -3161,10 +3212,10 @@
         <v>10.3</v>
       </c>
       <c r="D34">
-        <v>0.0083</v>
+        <v>0.0028</v>
       </c>
       <c r="E34">
-        <v>0.0134</v>
+        <v>0.00535</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -3178,10 +3229,10 @@
         <v>10.55</v>
       </c>
       <c r="D35">
-        <v>0.0063</v>
+        <v>0.0019</v>
       </c>
       <c r="E35">
-        <v>0.01485</v>
+        <v>0.0065</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -3195,10 +3246,10 @@
         <v>10.8</v>
       </c>
       <c r="D36">
-        <v>0.00525</v>
+        <v>0.00115</v>
       </c>
       <c r="E36">
-        <v>0.01715</v>
+        <v>0.008200000000000001</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -3212,10 +3263,10 @@
         <v>11.05</v>
       </c>
       <c r="D37">
-        <v>0.0042</v>
+        <v>0.0007</v>
       </c>
       <c r="E37">
-        <v>0.0186</v>
+        <v>0.0097</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3229,10 +3280,10 @@
         <v>11.3</v>
       </c>
       <c r="D38">
-        <v>0.00285</v>
+        <v>0.00055</v>
       </c>
       <c r="E38">
-        <v>0.02055</v>
+        <v>0.01145</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -3246,10 +3297,10 @@
         <v>11.55</v>
       </c>
       <c r="D39">
-        <v>0.0021</v>
+        <v>0.00045</v>
       </c>
       <c r="E39">
-        <v>0.0223</v>
+        <v>0.0132</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -3263,10 +3314,10 @@
         <v>11.8</v>
       </c>
       <c r="D40">
-        <v>0.0014</v>
+        <v>0.0003</v>
       </c>
       <c r="E40">
-        <v>0.0243</v>
+        <v>0.01545</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -3280,10 +3331,10 @@
         <v>12.05</v>
       </c>
       <c r="D41">
-        <v>0.0011</v>
+        <v>0.00015</v>
       </c>
       <c r="E41">
-        <v>0.0263</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -3297,10 +3348,10 @@
         <v>12.3</v>
       </c>
       <c r="D42">
-        <v>0.0008</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>0.0291</v>
+        <v>0.0199</v>
       </c>
     </row>
   </sheetData>
@@ -3310,7 +3361,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3332,13 +3383,13 @@
         <v>363</v>
       </c>
       <c r="B2">
-        <v>0.2648</v>
+        <v>0.3107</v>
       </c>
       <c r="C2">
-        <v>0.1905499999999999</v>
+        <v>0.2764</v>
       </c>
       <c r="D2">
-        <v>0.30465</v>
+        <v>0.4154</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -3346,13 +3397,13 @@
         <v>364</v>
       </c>
       <c r="B3">
-        <v>0.24115</v>
+        <v>0.34975</v>
       </c>
       <c r="C3">
-        <v>0.2003</v>
+        <v>0.32345</v>
       </c>
       <c r="D3">
-        <v>0.30035</v>
+        <v>0.4975</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3360,13 +3411,13 @@
         <v>365</v>
       </c>
       <c r="B4">
-        <v>24.53543451082598</v>
+        <v>-2094.563876428484</v>
       </c>
       <c r="C4">
-        <v>23.79098222453694</v>
+        <v>-4258.981809924959</v>
       </c>
       <c r="D4">
-        <v>30.28149215589269</v>
+        <v>82764293545.95332</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -3374,13 +3425,13 @@
         <v>366</v>
       </c>
       <c r="B5">
-        <v>0.2716</v>
+        <v>0.3263</v>
       </c>
       <c r="C5">
-        <v>0.1991</v>
+        <v>0.28955</v>
       </c>
       <c r="D5">
-        <v>0.30825</v>
+        <v>0.4346</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -3388,13 +3439,13 @@
         <v>367</v>
       </c>
       <c r="B6">
-        <v>0.25245</v>
+        <v>0.3739</v>
       </c>
       <c r="C6">
-        <v>0.2119</v>
+        <v>0.3397500000000001</v>
       </c>
       <c r="D6">
-        <v>0.3149</v>
+        <v>0.53185</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -3402,13 +3453,13 @@
         <v>368</v>
       </c>
       <c r="B7">
-        <v>25.2393772420323</v>
+        <v>-5571.026366859067</v>
       </c>
       <c r="C7">
-        <v>24.15059010492002</v>
+        <v>-11227.59836800903</v>
       </c>
       <c r="D7">
-        <v>31.08374281353895</v>
+        <v>57170283671.04326</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -3416,13 +3467,13 @@
         <v>369</v>
       </c>
       <c r="B8">
-        <v>0.3157</v>
+        <v>0.42485</v>
       </c>
       <c r="C8">
-        <v>0.2223</v>
+        <v>0.3045500000000001</v>
       </c>
       <c r="D8">
-        <v>0.3824499999999999</v>
+        <v>0.57675</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -3430,13 +3481,13 @@
         <v>370</v>
       </c>
       <c r="B9">
-        <v>0.34235</v>
+        <v>0.5414</v>
       </c>
       <c r="C9">
-        <v>0.2743000000000001</v>
+        <v>0.4076000000000001</v>
       </c>
       <c r="D9">
-        <v>0.4357</v>
+        <v>0.7767999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -3444,13 +3495,13 @@
         <v>371</v>
       </c>
       <c r="B10">
-        <v>30.82581548964391</v>
+        <v>-110758700.5515297</v>
       </c>
       <c r="C10">
-        <v>25.03251528537221</v>
+        <v>-221517531.7943307</v>
       </c>
       <c r="D10">
-        <v>39.93914663241513</v>
+        <v>207930966432232.6</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -3458,13 +3509,13 @@
         <v>372</v>
       </c>
       <c r="B11">
-        <v>0.327</v>
+        <v>0.33855</v>
       </c>
       <c r="C11">
-        <v>0.2769</v>
+        <v>0.3111</v>
       </c>
       <c r="D11">
-        <v>0.378</v>
+        <v>0.44615</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -3472,13 +3523,13 @@
         <v>373</v>
       </c>
       <c r="B12">
-        <v>0.24715</v>
+        <v>0.2762</v>
       </c>
       <c r="C12">
-        <v>0.20925</v>
+        <v>0.2284</v>
       </c>
       <c r="D12">
-        <v>0.31335</v>
+        <v>0.38245</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -3486,13 +3537,13 @@
         <v>374</v>
       </c>
       <c r="B13">
-        <v>0.3129</v>
+        <v>0.38515</v>
       </c>
       <c r="C13">
-        <v>0.2708</v>
+        <v>0.3593</v>
       </c>
       <c r="D13">
-        <v>0.387</v>
+        <v>0.5373</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -3500,13 +3551,13 @@
         <v>375</v>
       </c>
       <c r="B14">
-        <v>0.2604</v>
+        <v>0.36245</v>
       </c>
       <c r="C14">
-        <v>0.2135500000000001</v>
+        <v>0.34085</v>
       </c>
       <c r="D14">
-        <v>0.34985</v>
+        <v>0.5379</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -3514,13 +3565,13 @@
         <v>376</v>
       </c>
       <c r="B15">
-        <v>37.26481046992132</v>
+        <v>55.15383779591493</v>
       </c>
       <c r="C15">
-        <v>31.42019326213387</v>
+        <v>21.07903713454337</v>
       </c>
       <c r="D15">
-        <v>50.10493958944761</v>
+        <v>81.2488922616362</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -3528,13 +3579,13 @@
         <v>377</v>
       </c>
       <c r="B16">
-        <v>31.41768304365029</v>
+        <v>33.06163961284898</v>
       </c>
       <c r="C16">
-        <v>30.93384353684846</v>
+        <v>32.42867969046616</v>
       </c>
       <c r="D16">
-        <v>34.5984262237321</v>
+        <v>35.1173339588311</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -3542,13 +3593,13 @@
         <v>378</v>
       </c>
       <c r="B17">
-        <v>0.0068</v>
+        <v>0.0156</v>
       </c>
       <c r="C17">
-        <v>-0.0024999999999999</v>
+        <v>0.0011999999999999</v>
       </c>
       <c r="D17">
-        <v>0.0126</v>
+        <v>0.0292</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -3556,13 +3607,13 @@
         <v>379</v>
       </c>
       <c r="B18">
-        <v>0.0113</v>
+        <v>0.02415</v>
       </c>
       <c r="C18">
-        <v>0.0016</v>
+        <v>0.0033</v>
       </c>
       <c r="D18">
-        <v>0.0196</v>
+        <v>0.0443</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -3570,13 +3621,13 @@
         <v>380</v>
       </c>
       <c r="B19">
-        <v>0.7039427312063111</v>
+        <v>-3476.462490430584</v>
       </c>
       <c r="C19">
-        <v>-0.0400372126022809</v>
+        <v>-3396329840.932967</v>
       </c>
       <c r="D19">
-        <v>1.29889576976096</v>
+        <v>444849410.2697247</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -3584,13 +3635,13 @@
         <v>381</v>
       </c>
       <c r="B20">
-        <v>0.0509</v>
+        <v>0.11415</v>
       </c>
       <c r="C20">
-        <v>0.00245</v>
+        <v>-0.0117499999999999</v>
       </c>
       <c r="D20">
-        <v>0.10095</v>
+        <v>0.2013</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -3598,13 +3649,13 @@
         <v>382</v>
       </c>
       <c r="B21">
-        <v>0.1011999999999999</v>
+        <v>0.19165</v>
       </c>
       <c r="C21">
-        <v>0.0372</v>
+        <v>0.03225</v>
       </c>
       <c r="D21">
-        <v>0.1723999999999999</v>
+        <v>0.3383</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -3612,13 +3663,13 @@
         <v>383</v>
       </c>
       <c r="B22">
-        <v>6.290380978817925</v>
+        <v>-110756605.9876532</v>
       </c>
       <c r="C22">
-        <v>-0.2297438944255265</v>
+        <v>-249574302.5617398</v>
       </c>
       <c r="D22">
-        <v>11.81115210738872</v>
+        <v>50954209072032.45</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -3626,13 +3677,13 @@
         <v>384</v>
       </c>
       <c r="B23">
-        <v>14.88099010578472</v>
+        <v>2.411588676719129E-05</v>
       </c>
       <c r="C23">
-        <v>9.533037435279541</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>28.38790795089076</v>
+        <v>4.823177353438248E-05</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -3640,13 +3691,13 @@
         <v>385</v>
       </c>
       <c r="B24">
-        <v>8.671513634876966</v>
+        <v>0.0012008485320559</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>15.74394110066424</v>
+        <v>0.0024016970641118</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -3654,13 +3705,13 @@
         <v>386</v>
       </c>
       <c r="B25">
-        <v>35.63317440979731</v>
+        <v>0.0030417212026538</v>
       </c>
       <c r="C25">
-        <v>19.47126950014145</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>55.67825912561951</v>
+        <v>0.0060834424053076</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -3668,13 +3719,13 @@
         <v>387</v>
       </c>
       <c r="B26">
-        <v>40.814321849541</v>
+        <v>99.99573331437853</v>
       </c>
       <c r="C26">
-        <v>6.836499781635396</v>
+        <v>99.99146662875704</v>
       </c>
       <c r="D26">
-        <v>56.57602760597069</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -3682,13 +3733,13 @@
         <v>388</v>
       </c>
       <c r="B27">
-        <v>285.5941455781351</v>
+        <v>9468.799373351174</v>
       </c>
       <c r="C27">
-        <v>-94.39331446743574</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>509.8016243673768</v>
+        <v>18937.57385893837</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -3696,13 +3747,13 @@
         <v>389</v>
       </c>
       <c r="B28">
-        <v>405.5574961455612</v>
+        <v>0.0009507363069536</v>
       </c>
       <c r="C28">
-        <v>-324.9331437562977</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>731.0363720671497</v>
+        <v>0.0019014726139072</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -3710,13 +3761,13 @@
         <v>390</v>
       </c>
       <c r="B29">
-        <v>70.23801978843055</v>
+        <v>0.0008468706934859</v>
       </c>
       <c r="C29">
-        <v>43.22418409821846</v>
+        <v>0</v>
       </c>
       <c r="D29">
-        <v>80.93392512944098</v>
+        <v>0.0016937413869719</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -3724,7 +3775,13 @@
         <v>391</v>
       </c>
       <c r="B30">
-        <v>5.94991274725859</v>
+        <v>17612469273.93737</v>
+      </c>
+      <c r="C30">
+        <v>-6.752294116090375E+24</v>
+      </c>
+      <c r="D30">
+        <v>35224938350.32559</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -3732,7 +3789,13 @@
         <v>392</v>
       </c>
       <c r="B31">
-        <v>31.89828026046504</v>
+        <v>5340184.341112689</v>
+      </c>
+      <c r="C31">
+        <v>-1.846816488240213E+21</v>
+      </c>
+      <c r="D31">
+        <v>10680236.95187508</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -3740,7 +3803,13 @@
         <v>393</v>
       </c>
       <c r="B32">
-        <v>21.78079389627244</v>
+        <v>99.99995176822648</v>
+      </c>
+      <c r="C32">
+        <v>99.99990353645292</v>
+      </c>
+      <c r="D32">
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3748,7 +3817,7 @@
         <v>394</v>
       </c>
       <c r="B33">
-        <v>0.0031199435892336</v>
+        <v>-41881.30327002463</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3756,7 +3825,31 @@
         <v>395</v>
       </c>
       <c r="B34">
-        <v>0.0030248692327107</v>
+        <v>31.89828026046504</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>396</v>
+      </c>
+      <c r="B35">
+        <v>21.78079389627244</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>397</v>
+      </c>
+      <c r="B36">
+        <v>0.0032723501493574</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>398</v>
+      </c>
+      <c r="B37">
+        <v>0.0033721279446367</v>
       </c>
     </row>
   </sheetData>
@@ -3779,7 +3872,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B2">
         <v>0.2405</v>
@@ -3787,7 +3880,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B3">
         <v>0.20645</v>
@@ -3795,7 +3888,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B4">
         <v>52.31568005986517</v>
@@ -3803,7 +3896,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B5">
         <v>148.3740149659404</v>
@@ -27799,22 +27892,22 @@
         <v>52</v>
       </c>
       <c r="D2">
-        <v>12.31723954374397</v>
+        <v>12.17256735234501</v>
       </c>
       <c r="E2">
-        <v>13.87949119134747</v>
+        <v>14.32066336779984</v>
       </c>
       <c r="F2">
-        <v>12.95099886120318</v>
+        <v>13.04398641385144</v>
       </c>
       <c r="G2">
-        <v>0.8441012285016006</v>
+        <v>0.7463664783668131</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1.961781892117911E-07</v>
+        <v>9.676777806647184E-07</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -27837,22 +27930,22 @@
         <v>52</v>
       </c>
       <c r="D3">
-        <v>12.01671507761583</v>
+        <v>11.85336645414481</v>
       </c>
       <c r="E3">
-        <v>13.96952963712022</v>
+        <v>14.39202538150051</v>
       </c>
       <c r="F3">
-        <v>12.80891422443986</v>
+        <v>12.88322534501604</v>
       </c>
       <c r="G3">
-        <v>0.8955304312806546</v>
+        <v>0.7759218955353256</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>0.0559723041593834</v>
+        <v>0.0312909222073569</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -27875,22 +27968,22 @@
         <v>52</v>
       </c>
       <c r="D4">
-        <v>12.10561718135472</v>
+        <v>11.9362194729544</v>
       </c>
       <c r="E4">
-        <v>14.44899465275998</v>
+        <v>14.86544131221098</v>
       </c>
       <c r="F4">
-        <v>13.05625615754355</v>
+        <v>13.12451819319043</v>
       </c>
       <c r="G4">
-        <v>0.9376059201668934</v>
+        <v>0.8619925002311357</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>0.0113061333329902</v>
+        <v>0.0136585070231802</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -27913,22 +28006,22 @@
         <v>52</v>
       </c>
       <c r="D5">
-        <v>12.01870067458408</v>
+        <v>11.87338449135836</v>
       </c>
       <c r="E5">
-        <v>14.75264105789021</v>
+        <v>15.19316924251582</v>
       </c>
       <c r="F5">
-        <v>13.12777948013771</v>
+        <v>13.2201230409592</v>
       </c>
       <c r="G5">
-        <v>0.9796788521266264</v>
+        <v>0.9528741108949064</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
       </c>
       <c r="I5">
-        <v>0.0029553964210722</v>
+        <v>0.0002450761742959</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -27951,22 +28044,22 @@
         <v>52</v>
       </c>
       <c r="D6">
-        <v>11.95620329346106</v>
+        <v>11.90885846309727</v>
       </c>
       <c r="E6">
-        <v>15.08070658866808</v>
+        <v>15.6192061261556</v>
       </c>
       <c r="F6">
-        <v>13.2237219283795</v>
+        <v>13.41403684206291</v>
       </c>
       <c r="G6">
-        <v>0.9994961831765166</v>
+        <v>1.005002120146997</v>
       </c>
       <c r="H6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>0.0004100063223578</v>
+        <v>3.707142992104039E-05</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -27989,22 +28082,22 @@
         <v>52</v>
       </c>
       <c r="D7">
-        <v>11.90034478965944</v>
+        <v>11.82752854502258</v>
       </c>
       <c r="E7">
-        <v>15.41541099676734</v>
+        <v>15.92843911998178</v>
       </c>
       <c r="F7">
-        <v>13.32630325394268</v>
+        <v>13.49114675335302</v>
       </c>
       <c r="G7">
-        <v>1.005203026136796</v>
+        <v>1.007923002404729</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0.0002447272112527</v>
+        <v>7.477398576676402E-05</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -28039,7 +28132,7 @@
         <v>257</v>
       </c>
       <c r="B2">
-        <v>0.0559723041593834</v>
+        <v>0.0312909222073569</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -28047,7 +28140,7 @@
         <v>258</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1.53350226418298E-232</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -28063,7 +28156,7 @@
         <v>260</v>
       </c>
       <c r="B5">
-        <v>0.9879867416903756</v>
+        <v>0.9602771826033332</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -28071,7 +28164,7 @@
         <v>261</v>
       </c>
       <c r="B6">
-        <v>0.7459676639764559</v>
+        <v>0.8329731262226052</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -28079,7 +28172,7 @@
         <v>262</v>
       </c>
       <c r="B7">
-        <v>0.996166125115002</v>
+        <v>0.9245382459474112</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -28087,7 +28180,7 @@
         <v>263</v>
       </c>
       <c r="B8">
-        <v>0.1078991572050148</v>
+        <v>3.076252835122526E-06</v>
       </c>
     </row>
   </sheetData>
@@ -28119,13 +28212,13 @@
         <v>267</v>
       </c>
       <c r="B2">
-        <v>0.0220129519801578</v>
+        <v>0.0230593828594906</v>
       </c>
       <c r="C2">
-        <v>0.0575970757040603</v>
+        <v>0.0466221639234013</v>
       </c>
       <c r="D2">
-        <v>0.0821759114770777</v>
+        <v>0.0835148388900239</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -28133,13 +28226,13 @@
         <v>268</v>
       </c>
       <c r="B3">
-        <v>0.1118020071995374</v>
+        <v>0.061661134992728</v>
       </c>
       <c r="C3">
-        <v>0.1993294540964628</v>
+        <v>0.079383058161742</v>
       </c>
       <c r="D3">
-        <v>0.3283453050693037</v>
+        <v>0.1469123321339287</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -28147,13 +28240,13 @@
         <v>269</v>
       </c>
       <c r="B4">
-        <v>0.0220129519801578</v>
+        <v>0.0230593828594906</v>
       </c>
       <c r="C4">
-        <v>0.0575970757040603</v>
+        <v>0.0466221639234013</v>
       </c>
       <c r="D4">
-        <v>0.0821759114770777</v>
+        <v>0.0835148388900239</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -28161,13 +28254,13 @@
         <v>270</v>
       </c>
       <c r="B5">
-        <v>-0.0164824184500533</v>
+        <v>-0.001422573557893</v>
       </c>
       <c r="C5">
-        <v>0.04981159927988</v>
+        <v>0.0714795958784846</v>
       </c>
       <c r="D5">
-        <v>0.08414794260844979</v>
+        <v>0.1255093777299399</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -28175,13 +28268,13 @@
         <v>271</v>
       </c>
       <c r="B6">
-        <v>-5.341417713641398</v>
+        <v>13.93795449584983</v>
       </c>
       <c r="C6">
-        <v>15.29254232419382</v>
+        <v>34.85779849977312</v>
       </c>
       <c r="D6">
-        <v>30.47205515708366</v>
+        <v>47.61471131682272</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -28189,13 +28282,13 @@
         <v>272</v>
       </c>
       <c r="B7">
-        <v>-0.0031250317659136</v>
+        <v>-0.0024201902037544</v>
       </c>
       <c r="C7">
-        <v>-0.0012099172636955</v>
+        <v>-0.0002925536451941</v>
       </c>
       <c r="D7">
-        <v>0.0007734156417453</v>
+        <v>0.0022918358523219</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -28203,13 +28296,13 @@
         <v>273</v>
       </c>
       <c r="B8">
-        <v>-0.0365292238257445</v>
+        <v>0.0164194698506899</v>
       </c>
       <c r="C8">
-        <v>0.3062162572993613</v>
+        <v>0.316556592062593</v>
       </c>
       <c r="D8">
-        <v>0.6917782734703539</v>
+        <v>0.7049805723868801</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -28217,13 +28310,13 @@
         <v>274</v>
       </c>
       <c r="B9">
-        <v>-0.2734996021874047</v>
+        <v>-0.0941002650966771</v>
       </c>
       <c r="C9">
-        <v>0.4388340258290752</v>
+        <v>0.5290271025417446</v>
       </c>
       <c r="D9">
-        <v>1.113492371448088</v>
+        <v>1.283106221437569</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -28231,13 +28324,13 @@
         <v>275</v>
       </c>
       <c r="B10">
-        <v>-93.60502983695064</v>
+        <v>-61.43952577576145</v>
       </c>
       <c r="C10">
-        <v>7.234831382796857</v>
+        <v>44.9420408440044</v>
       </c>
       <c r="D10">
-        <v>132.5221325282151</v>
+        <v>121.3334553605959</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -28245,13 +28338,13 @@
         <v>276</v>
       </c>
       <c r="B11">
-        <v>-0.0363796402985956</v>
+        <v>-0.0271244544496328</v>
       </c>
       <c r="C11">
-        <v>-0.0175800739744947</v>
+        <v>-0.0013098618013235</v>
       </c>
       <c r="D11">
-        <v>0.0103469811386898</v>
+        <v>0.0209981921980148</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -28259,13 +28352,13 @@
         <v>277</v>
       </c>
       <c r="B12">
-        <v>-0.5296111094079572</v>
+        <v>-0.5654611366391767</v>
       </c>
       <c r="C12">
-        <v>-0.12420211955139</v>
+        <v>-0.1217703147582797</v>
       </c>
       <c r="D12">
-        <v>0.2509814560418417</v>
+        <v>0.2701633783821436</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -28273,13 +28366,13 @@
         <v>278</v>
       </c>
       <c r="B13">
-        <v>-0.9422152917632278</v>
+        <v>-0.9584962051831264</v>
       </c>
       <c r="C13">
-        <v>-0.0510049263396294</v>
+        <v>-0.0253497617875721</v>
       </c>
       <c r="D13">
-        <v>0.7166427399668879</v>
+        <v>0.7467144269288195</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -28287,13 +28380,13 @@
         <v>279</v>
       </c>
       <c r="B14">
-        <v>-109.5642906926216</v>
+        <v>-105.4862861154182</v>
       </c>
       <c r="C14">
-        <v>-10.24387449946999</v>
+        <v>-23.33956898933793</v>
       </c>
       <c r="D14">
-        <v>112.6435258486871</v>
+        <v>92.83886234052066</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -28301,13 +28394,13 @@
         <v>280</v>
       </c>
       <c r="B15">
-        <v>-0.0431079579565937</v>
+        <v>-0.0371333127564079</v>
       </c>
       <c r="C15">
-        <v>-0.0234611824393953</v>
+        <v>-0.0160873808522476</v>
       </c>
       <c r="D15">
-        <v>0.0119680653847869</v>
+        <v>0.011674043185748</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -28315,13 +28408,13 @@
         <v>281</v>
       </c>
       <c r="B16">
-        <v>-0.344863720931649</v>
+        <v>-0.2863148084214579</v>
       </c>
       <c r="C16">
-        <v>0.0058303340623681</v>
+        <v>0.0145915485299101</v>
       </c>
       <c r="D16">
-        <v>0.3147533469839956</v>
+        <v>0.4339683820885656</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -28329,13 +28422,13 @@
         <v>282</v>
       </c>
       <c r="B17">
-        <v>-0.8603104402954707</v>
+        <v>-0.9754470963888566</v>
       </c>
       <c r="C17">
-        <v>-0.1587192626338701</v>
+        <v>-0.2031723567147852</v>
       </c>
       <c r="D17">
-        <v>0.6738959726395306</v>
+        <v>0.6271573685204861</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -28343,13 +28436,13 @@
         <v>283</v>
       </c>
       <c r="B18">
-        <v>-194.3909760116757</v>
+        <v>-128.6331050209795</v>
       </c>
       <c r="C18">
-        <v>-90.17957898161042</v>
+        <v>-14.0805826099547</v>
       </c>
       <c r="D18">
-        <v>15.82283387366294</v>
+        <v>82.03269831978075</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -28357,13 +28450,13 @@
         <v>284</v>
       </c>
       <c r="B19">
-        <v>-0.0525282082567274</v>
+        <v>-0.0485147212027431</v>
       </c>
       <c r="C19">
-        <v>-0.0322965744878888</v>
+        <v>-0.0307313133497251</v>
       </c>
       <c r="D19">
-        <v>-0.0025658079369072</v>
+        <v>-0.0062975716276822</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -28371,13 +28464,13 @@
         <v>285</v>
       </c>
       <c r="B20">
-        <v>-0.2979348028993886</v>
+        <v>-0.2762159923191306</v>
       </c>
       <c r="C20">
-        <v>-0.0442489433112968</v>
+        <v>-0.0811314026504157</v>
       </c>
       <c r="D20">
-        <v>0.1441496647972949</v>
+        <v>0.1024641803697696</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -28385,13 +28478,13 @@
         <v>286</v>
       </c>
       <c r="B21">
-        <v>-0.4072910196661679</v>
+        <v>-0.5105598153566</v>
       </c>
       <c r="C21">
-        <v>-0.0456726750775331</v>
+        <v>-0.1063775491762813</v>
       </c>
       <c r="D21">
-        <v>0.3084965608843515</v>
+        <v>0.207397290736667</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -28399,13 +28492,13 @@
         <v>287</v>
       </c>
       <c r="B22">
-        <v>-160.8237668437943</v>
+        <v>-53.34029988225009</v>
       </c>
       <c r="C22">
-        <v>-57.3976055206734</v>
+        <v>23.56309685469024</v>
       </c>
       <c r="D22">
-        <v>40.79111632613531</v>
+        <v>83.79743518220653</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -28413,13 +28506,13 @@
         <v>288</v>
       </c>
       <c r="B23">
-        <v>-0.0536654371734015</v>
+        <v>-0.0514032924880218</v>
       </c>
       <c r="C23">
-        <v>-0.0308332905542092</v>
+        <v>-0.0290642700292457</v>
       </c>
       <c r="D23">
-        <v>-0.0031930245454782</v>
+        <v>-0.0062368604930251</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -28427,13 +28520,13 @@
         <v>289</v>
       </c>
       <c r="B24">
-        <v>-0.2853141303891852</v>
+        <v>-0.2617491153613754</v>
       </c>
       <c r="C24">
-        <v>-0.0367036089960932</v>
+        <v>-0.0923704860426421</v>
       </c>
       <c r="D24">
-        <v>0.170859171566036</v>
+        <v>0.1178345058087008</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -28441,13 +28534,13 @@
         <v>290</v>
       </c>
       <c r="B25">
-        <v>-0.2978518305757773</v>
+        <v>-0.2475780599710562</v>
       </c>
       <c r="C25">
-        <v>-0.0542601885069263</v>
+        <v>-0.051667060058603</v>
       </c>
       <c r="D25">
-        <v>0.1675445238881066</v>
+        <v>0.2551246677705699</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -28455,13 +28548,13 @@
         <v>291</v>
       </c>
       <c r="B26">
-        <v>-87.66682638898321</v>
+        <v>1.528516190845039</v>
       </c>
       <c r="C26">
-        <v>-13.41672352016079</v>
+        <v>62.30598361937489</v>
       </c>
       <c r="D26">
-        <v>73.6916034982923</v>
+        <v>122.2400421686716</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -28469,13 +28562,13 @@
         <v>292</v>
       </c>
       <c r="B27">
-        <v>-0.0424818811235572</v>
+        <v>-0.0379832202375733</v>
       </c>
       <c r="C27">
-        <v>-0.0209622562523362</v>
+        <v>-0.0189370866247148</v>
       </c>
       <c r="D27">
-        <v>0.0063205754672177</v>
+        <v>0.001785944757952</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -28483,13 +28576,13 @@
         <v>293</v>
       </c>
       <c r="B28">
-        <v>-0.2531378767877441</v>
+        <v>-0.2397761708551044</v>
       </c>
       <c r="C28">
-        <v>-0.0478821161681045</v>
+        <v>-0.1086556841785406</v>
       </c>
       <c r="D28">
-        <v>0.1081173493473235</v>
+        <v>-0.0043761011808898</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -28497,13 +28590,13 @@
         <v>294</v>
       </c>
       <c r="B29">
-        <v>-0.2552611392246665</v>
+        <v>-0.2799846376667973</v>
       </c>
       <c r="C29">
-        <v>-0.1101969929432576</v>
+        <v>-0.1193429302270634</v>
       </c>
       <c r="D29">
-        <v>0.0444747265994615</v>
+        <v>0.07699165808316109</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -28511,13 +28604,13 @@
         <v>295</v>
       </c>
       <c r="B30">
-        <v>-33.99286262712005</v>
+        <v>16.75725999207226</v>
       </c>
       <c r="C30">
-        <v>14.46032297516378</v>
+        <v>62.68484851659193</v>
       </c>
       <c r="D30">
-        <v>85.24940678638073</v>
+        <v>128.0446550813975</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -28525,13 +28618,13 @@
         <v>296</v>
       </c>
       <c r="B31">
-        <v>-0.0304183756306734</v>
+        <v>-0.0252731442959393</v>
       </c>
       <c r="C31">
-        <v>-0.0117831317294659</v>
+        <v>-0.0103487478259911</v>
       </c>
       <c r="D31">
-        <v>0.0124702560884935</v>
+        <v>0.0078052312056977</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -28539,13 +28632,13 @@
         <v>297</v>
       </c>
       <c r="B32">
-        <v>-0.2342368201230044</v>
+        <v>-0.2067232981593788</v>
       </c>
       <c r="C32">
-        <v>-0.0557421726272658</v>
+        <v>-0.1035159184684966</v>
       </c>
       <c r="D32">
-        <v>0.0899439477147732</v>
+        <v>-0.0028759486474579</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -28553,13 +28646,13 @@
         <v>298</v>
       </c>
       <c r="B33">
-        <v>-0.1666858469898699</v>
+        <v>-0.211461362030848</v>
       </c>
       <c r="C33">
-        <v>-0.06609853850607419</v>
+        <v>-0.0869757313221844</v>
       </c>
       <c r="D33">
-        <v>0.0604560734685235</v>
+        <v>0.027247256598769</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -28567,13 +28660,13 @@
         <v>299</v>
       </c>
       <c r="B34">
-        <v>-13.58361498562164</v>
+        <v>2.015694677782477</v>
       </c>
       <c r="C34">
-        <v>24.79200799182408</v>
+        <v>43.15167982639244</v>
       </c>
       <c r="D34">
-        <v>79.40931445587297</v>
+        <v>99.60224266886151</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -28581,13 +28674,13 @@
         <v>300</v>
       </c>
       <c r="B35">
-        <v>-0.0204461377220727</v>
+        <v>-0.0150346463627311</v>
       </c>
       <c r="C35">
-        <v>-0.0053009451700465</v>
+        <v>-0.0047625622798913</v>
       </c>
       <c r="D35">
-        <v>0.0149431153094812</v>
+        <v>0.00917910199917</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -28595,13 +28688,13 @@
         <v>301</v>
       </c>
       <c r="B36">
-        <v>-0.2186926309429426</v>
+        <v>-0.1933694134951277</v>
       </c>
       <c r="C36">
-        <v>-0.06277768593887249</v>
+        <v>-0.0971048574447789</v>
       </c>
       <c r="D36">
-        <v>0.0757612634899034</v>
+        <v>-0.0188075635840666</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -28609,13 +28702,13 @@
         <v>302</v>
       </c>
       <c r="B37">
-        <v>-0.08534163935375751</v>
+        <v>-0.1336907390435502</v>
       </c>
       <c r="C37">
-        <v>-0.0149624553927555</v>
+        <v>-0.0294477097115337</v>
       </c>
       <c r="D37">
-        <v>0.0768099432531885</v>
+        <v>0.0594103097216169</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -28623,13 +28716,13 @@
         <v>303</v>
       </c>
       <c r="B38">
-        <v>-10.41253052359276</v>
+        <v>-13.39548634730399</v>
       </c>
       <c r="C38">
-        <v>23.79626152316828</v>
+        <v>21.8383274758884</v>
       </c>
       <c r="D38">
-        <v>61.32960122215232</v>
+        <v>59.05188817475008</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -28637,13 +28730,13 @@
         <v>304</v>
       </c>
       <c r="B39">
-        <v>-0.0170507393280847</v>
+        <v>-0.0119762878814608</v>
       </c>
       <c r="C39">
-        <v>-0.0022016060064308</v>
+        <v>-0.0023765995677488</v>
       </c>
       <c r="D39">
-        <v>0.0141103248975173</v>
+        <v>0.0077351831841714</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -28651,13 +28744,13 @@
         <v>305</v>
       </c>
       <c r="B40">
-        <v>-0.1927112010376264</v>
+        <v>-0.1525767687499875</v>
       </c>
       <c r="C40">
-        <v>-0.0580487132297087</v>
+        <v>-0.0721288324770472</v>
       </c>
       <c r="D40">
-        <v>0.0609059836362788</v>
+        <v>-0.0151436653003143</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -28665,13 +28758,13 @@
         <v>306</v>
       </c>
       <c r="B41">
-        <v>-0.0569469847459309</v>
+        <v>-0.0696151944794175</v>
       </c>
       <c r="C41">
-        <v>0.0039227248911569</v>
+        <v>-5.506211864746494E-05</v>
       </c>
       <c r="D41">
-        <v>0.07400893743908001</v>
+        <v>0.0745670505042831</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -28679,13 +28772,13 @@
         <v>307</v>
       </c>
       <c r="B42">
-        <v>-13.53774782310306</v>
+        <v>-23.86914436089989</v>
       </c>
       <c r="C42">
-        <v>17.71261399260089</v>
+        <v>5.449159254287944</v>
       </c>
       <c r="D42">
-        <v>47.25885998582471</v>
+        <v>34.69287975391549</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -28693,13 +28786,13 @@
         <v>308</v>
       </c>
       <c r="B43">
-        <v>-0.0147545513075159</v>
+        <v>-0.0112060341570362</v>
       </c>
       <c r="C43">
-        <v>-0.0015601946658637</v>
+        <v>-0.0020271943581669</v>
       </c>
       <c r="D43">
-        <v>0.0111409577754987</v>
+        <v>0.0057993361075883</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -28707,13 +28800,13 @@
         <v>309</v>
       </c>
       <c r="B44">
-        <v>-0.1678016800483035</v>
+        <v>-0.1100370008288207</v>
       </c>
       <c r="C44">
-        <v>-0.0514976642152133</v>
+        <v>-0.046940529863347</v>
       </c>
       <c r="D44">
-        <v>0.0514820542842168</v>
+        <v>-0.001635578933114</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -28721,13 +28814,13 @@
         <v>310</v>
       </c>
       <c r="B45">
-        <v>-0.0456173176249218</v>
+        <v>-0.06665429877663361</v>
       </c>
       <c r="C45">
-        <v>0.0013189927706312</v>
+        <v>-0.0011790340179682</v>
       </c>
       <c r="D45">
-        <v>0.0504564736678648</v>
+        <v>0.0422864822674101</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -28735,13 +28828,13 @@
         <v>311</v>
       </c>
       <c r="B46">
-        <v>-15.3595551315119</v>
+        <v>-27.53056228751601</v>
       </c>
       <c r="C46">
-        <v>11.11782144740361</v>
+        <v>-3.754543922008006</v>
       </c>
       <c r="D46">
-        <v>35.1971909095126</v>
+        <v>22.70788103064022</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -28749,13 +28842,13 @@
         <v>312</v>
       </c>
       <c r="B47">
-        <v>-0.0141059967186471</v>
+        <v>-0.0108776898579514</v>
       </c>
       <c r="C47">
-        <v>-0.002119912949419</v>
+        <v>-0.0026908180263826</v>
       </c>
       <c r="D47">
-        <v>0.007922999476865301</v>
+        <v>0.0032829219762217</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -28763,13 +28856,13 @@
         <v>313</v>
       </c>
       <c r="B48">
-        <v>-0.1473246634164245</v>
+        <v>-0.0808681922724081</v>
       </c>
       <c r="C48">
-        <v>-0.044853197203204</v>
+        <v>-0.0278906467207164</v>
       </c>
       <c r="D48">
-        <v>0.0411030317040683</v>
+        <v>0.0090755392121136</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -28777,13 +28870,13 @@
         <v>314</v>
       </c>
       <c r="B49">
-        <v>-0.0471251705309423</v>
+        <v>-0.0636609524893629</v>
       </c>
       <c r="C49">
-        <v>-0.0012295128391159</v>
+        <v>-0.0038577188135254</v>
       </c>
       <c r="D49">
-        <v>0.0343799093884666</v>
+        <v>0.0295028085801644</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -28791,13 +28884,13 @@
         <v>315</v>
       </c>
       <c r="B50">
-        <v>-15.10583386501554</v>
+        <v>-25.57550114453377</v>
       </c>
       <c r="C50">
-        <v>6.463123285862038</v>
+        <v>-5.395628036296092</v>
       </c>
       <c r="D50">
-        <v>27.46993362583092</v>
+        <v>14.18863231650174</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -28805,13 +28898,13 @@
         <v>316</v>
       </c>
       <c r="B51">
-        <v>-0.0136033353315265</v>
+        <v>-0.009764595679587</v>
       </c>
       <c r="C51">
-        <v>-0.0027717638282557</v>
+        <v>-0.0032187869165724</v>
       </c>
       <c r="D51">
-        <v>0.0053310322888564</v>
+        <v>0.0018565237556521</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -28819,13 +28912,13 @@
         <v>317</v>
       </c>
       <c r="B52">
-        <v>-0.1280637885372794</v>
+        <v>-0.0654778095337446</v>
       </c>
       <c r="C52">
-        <v>-0.0396434341184137</v>
+        <v>-0.0178985784715391</v>
       </c>
       <c r="D52">
-        <v>0.0332728930423242</v>
+        <v>0.0135658896606771</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -28833,13 +28926,13 @@
         <v>318</v>
       </c>
       <c r="B53">
-        <v>-0.0428074275384981</v>
+        <v>-0.0556613767085695</v>
       </c>
       <c r="C53">
-        <v>-0.0035128418425254</v>
+        <v>-0.0064447053373182</v>
       </c>
       <c r="D53">
-        <v>0.0223734837652544</v>
+        <v>0.0203468177550984</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -28847,13 +28940,13 @@
         <v>319</v>
       </c>
       <c r="B54">
-        <v>-11.95220134400972</v>
+        <v>-18.55119513096622</v>
       </c>
       <c r="C54">
-        <v>4.136024375884599</v>
+        <v>-2.391622509653396</v>
       </c>
       <c r="D54">
-        <v>22.14517481719247</v>
+        <v>14.69290415075878</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -28861,13 +28954,13 @@
         <v>320</v>
       </c>
       <c r="B55">
-        <v>-0.0119994255462901</v>
+        <v>-0.0079268359620284</v>
       </c>
       <c r="C55">
-        <v>-0.0030837302479971</v>
+        <v>-0.0031604920112848</v>
       </c>
       <c r="D55">
-        <v>0.0040221188309852</v>
+        <v>0.0011722975531876</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -28875,13 +28968,13 @@
         <v>321</v>
       </c>
       <c r="B56">
-        <v>-0.1150699497369811</v>
+        <v>-0.0511097584214413</v>
       </c>
       <c r="C56">
-        <v>-0.0351191622012939</v>
+        <v>-0.0132215329917317</v>
       </c>
       <c r="D56">
-        <v>0.030050282863749</v>
+        <v>0.0160636813812294</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -28889,13 +28982,13 @@
         <v>322</v>
       </c>
       <c r="B57">
-        <v>-0.0360994301195206</v>
+        <v>-0.0444319101351109</v>
       </c>
       <c r="C57">
-        <v>-0.0058975865803716</v>
+        <v>-0.0093611285062735</v>
       </c>
       <c r="D57">
-        <v>0.0150556140038291</v>
+        <v>0.0159090563716958</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -28903,13 +28996,13 @@
         <v>323</v>
       </c>
       <c r="B58">
-        <v>-8.921142361706149</v>
+        <v>-11.37275132316119</v>
       </c>
       <c r="C58">
-        <v>3.410580043688902</v>
+        <v>1.39176015501413</v>
       </c>
       <c r="D58">
-        <v>19.54163457251583</v>
+        <v>14.85575217430523</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -28917,13 +29010,13 @@
         <v>324</v>
       </c>
       <c r="B59">
-        <v>-0.0102965951434716</v>
+        <v>-0.00593808356312</v>
       </c>
       <c r="C59">
-        <v>-0.0030209441445786</v>
+        <v>-0.0025842720196632</v>
       </c>
       <c r="D59">
-        <v>0.0031767463542691</v>
+        <v>0.0013349131048961</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -28931,13 +29024,13 @@
         <v>325</v>
       </c>
       <c r="B60">
-        <v>-0.1027142264408473</v>
+        <v>-0.0411340162180715</v>
       </c>
       <c r="C60">
-        <v>-0.0315597715703665</v>
+        <v>-0.0117875577388299</v>
       </c>
       <c r="D60">
-        <v>0.0215160557179969</v>
+        <v>0.0118584842781577</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -28945,13 +29038,13 @@
         <v>326</v>
       </c>
       <c r="B61">
-        <v>-0.0306656572666062</v>
+        <v>-0.0322970176225238</v>
       </c>
       <c r="C61">
-        <v>-0.0073430734427969</v>
+        <v>-0.0107970203649473</v>
       </c>
       <c r="D61">
-        <v>0.0111845244856227</v>
+        <v>0.0114146452764393</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -28959,13 +29052,13 @@
         <v>327</v>
       </c>
       <c r="B62">
-        <v>-6.581788638064874</v>
+        <v>-6.80256769199616</v>
       </c>
       <c r="C62">
-        <v>3.403317047529938</v>
+        <v>3.664701166016767</v>
       </c>
       <c r="D62">
-        <v>18.74500613260557</v>
+        <v>12.7391836442816</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -28973,13 +29066,13 @@
         <v>328</v>
       </c>
       <c r="B63">
-        <v>-0.0089649675764076</v>
+        <v>-0.004152644170894</v>
       </c>
       <c r="C63">
-        <v>-0.0027262176182029</v>
+        <v>-0.0018137406774841</v>
       </c>
       <c r="D63">
-        <v>0.0027356363632662</v>
+        <v>0.0017511753430691</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -28987,13 +29080,13 @@
         <v>329</v>
       </c>
       <c r="B64">
-        <v>-0.0919725001438913</v>
+        <v>-0.0317681295230432</v>
       </c>
       <c r="C64">
-        <v>-0.0286064782660036</v>
+        <v>-0.0112792544174378</v>
       </c>
       <c r="D64">
-        <v>0.0212802069163934</v>
+        <v>0.009251483150018801</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -29001,13 +29094,13 @@
         <v>330</v>
       </c>
       <c r="B65">
-        <v>-0.0250271833670431</v>
+        <v>-0.0243901321910182</v>
       </c>
       <c r="C65">
-        <v>-0.0069963799987745</v>
+        <v>-0.008987660663061101</v>
       </c>
       <c r="D65">
-        <v>0.0098948702664431</v>
+        <v>0.010781377563801</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -29015,13 +29108,13 @@
         <v>331</v>
       </c>
       <c r="B66">
-        <v>-4.984997798467735</v>
+        <v>-5.670143823347173</v>
       </c>
       <c r="C66">
-        <v>3.518410536731235</v>
+        <v>4.052940901129775</v>
       </c>
       <c r="D66">
-        <v>16.71717748385183</v>
+        <v>10.53481481162321</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -29029,13 +29122,13 @@
         <v>332</v>
       </c>
       <c r="B67">
-        <v>-0.0076636414886686</v>
+        <v>-0.00289573486325</v>
       </c>
       <c r="C67">
-        <v>-0.0023476131937067</v>
+        <v>-0.0011166604533155</v>
       </c>
       <c r="D67">
-        <v>0.0024885676645071</v>
+        <v>0.0026702348584678</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -29043,13 +29136,13 @@
         <v>333</v>
       </c>
       <c r="B68">
-        <v>-0.0832426713578049</v>
+        <v>-0.0255228527240407</v>
       </c>
       <c r="C68">
-        <v>-0.0260188603568699</v>
+        <v>-0.0104088763230492</v>
       </c>
       <c r="D68">
-        <v>0.0186485789190647</v>
+        <v>0.008273388550184901</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -29057,13 +29150,13 @@
         <v>334</v>
       </c>
       <c r="B69">
-        <v>-0.0205045574972229</v>
+        <v>-0.0169565141779651</v>
       </c>
       <c r="C69">
-        <v>-0.0058561031446984</v>
+        <v>-0.0058091400774555</v>
       </c>
       <c r="D69">
-        <v>0.009783852550893901</v>
+        <v>0.0128498988908222</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -29071,13 +29164,13 @@
         <v>335</v>
       </c>
       <c r="B70">
-        <v>-4.036050390010161</v>
+        <v>-6.211642266137647</v>
       </c>
       <c r="C70">
-        <v>3.484903632242325</v>
+        <v>3.149273469106422</v>
       </c>
       <c r="D70">
-        <v>14.99442531568415</v>
+        <v>8.383189117712551</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -29085,13 +29178,13 @@
         <v>336</v>
       </c>
       <c r="B71">
-        <v>-0.0065617751136893</v>
+        <v>-0.0020130155791557</v>
       </c>
       <c r="C71">
-        <v>-0.0019934420377226</v>
+        <v>-0.0006391155803363</v>
       </c>
       <c r="D71">
-        <v>0.0023470839727275</v>
+        <v>0.0027041708263496</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -29099,13 +29192,13 @@
         <v>337</v>
       </c>
       <c r="B72">
-        <v>-0.074200448779635</v>
+        <v>-0.0192426685813009</v>
       </c>
       <c r="C72">
-        <v>-0.0235757755448638</v>
+        <v>-0.008705667029341601</v>
       </c>
       <c r="D72">
-        <v>0.0159685255562172</v>
+        <v>0.0091241937495769</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -29113,13 +29206,13 @@
         <v>338</v>
       </c>
       <c r="B73">
-        <v>-0.0170477050169806</v>
+        <v>-0.0126505859296677</v>
       </c>
       <c r="C73">
-        <v>-0.0047341034300663</v>
+        <v>-0.0030937792795211</v>
       </c>
       <c r="D73">
-        <v>0.0088995873148462</v>
+        <v>0.015101747641614</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -29127,13 +29220,13 @@
         <v>339</v>
       </c>
       <c r="B74">
-        <v>-3.74679476665565</v>
+        <v>-6.854456894084247</v>
       </c>
       <c r="C74">
-        <v>3.260061887015469</v>
+        <v>1.783547307506584</v>
       </c>
       <c r="D74">
-        <v>13.38807217507666</v>
+        <v>6.073467907614488</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -29141,13 +29234,13 @@
         <v>340</v>
       </c>
       <c r="B75">
-        <v>-0.0056734232040695</v>
+        <v>-0.001656814483135</v>
       </c>
       <c r="C75">
-        <v>-0.0017100759312807</v>
+        <v>-0.0003953151966167</v>
       </c>
       <c r="D75">
-        <v>0.0023986655780891</v>
+        <v>0.0022995304275289</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -29155,13 +29248,13 @@
         <v>341</v>
       </c>
       <c r="B76">
-        <v>-0.0650217257007354</v>
+        <v>-0.0154331642137886</v>
       </c>
       <c r="C76">
-        <v>-0.0212724823436318</v>
+        <v>-0.0065916476077858</v>
       </c>
       <c r="D76">
-        <v>0.0134629057737933</v>
+        <v>0.0101615381647712</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -29169,13 +29262,13 @@
         <v>342</v>
       </c>
       <c r="B77">
-        <v>-0.0148146609414312</v>
+        <v>-0.0086407802986755</v>
       </c>
       <c r="C77">
-        <v>-0.0038986686823361</v>
+        <v>-0.00146410194303</v>
       </c>
       <c r="D77">
-        <v>0.0077786164530823</v>
+        <v>0.0118769432170741</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -29183,13 +29276,13 @@
         <v>343</v>
       </c>
       <c r="B78">
-        <v>-3.411136327185172</v>
+        <v>-6.404587652762759</v>
       </c>
       <c r="C78">
-        <v>2.914333688449193</v>
+        <v>0.6239842269539193</v>
       </c>
       <c r="D78">
-        <v>11.3011185775007</v>
+        <v>4.328907898914762</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -29197,13 +29290,13 @@
         <v>344</v>
       </c>
       <c r="B79">
-        <v>-0.0049817673056266</v>
+        <v>-0.0014523509689208</v>
       </c>
       <c r="C79">
-        <v>-0.0014987868864349</v>
+        <v>-0.0003172452343273</v>
       </c>
       <c r="D79">
-        <v>0.0022595025006616</v>
+        <v>0.0018227520916616</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -29211,13 +29304,13 @@
         <v>345</v>
       </c>
       <c r="B80">
-        <v>-0.0584115653550364</v>
+        <v>-0.011832052892142</v>
       </c>
       <c r="C80">
-        <v>-0.0191218239700547</v>
+        <v>-0.0045993089282518</v>
       </c>
       <c r="D80">
-        <v>0.0129862925253256</v>
+        <v>0.0105299564322515</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -29225,13 +29318,13 @@
         <v>346</v>
       </c>
       <c r="B81">
-        <v>-0.0131467794057606</v>
+        <v>-0.0079084916640857</v>
       </c>
       <c r="C81">
-        <v>-0.0033044486725526</v>
+        <v>-0.000738727488139</v>
       </c>
       <c r="D81">
-        <v>0.0067177275416648</v>
+        <v>0.00922726813341</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -29239,13 +29332,13 @@
         <v>347</v>
       </c>
       <c r="B82">
-        <v>-2.85553211544765</v>
+        <v>-5.306502704647984</v>
       </c>
       <c r="C82">
-        <v>2.539567251532833</v>
+        <v>-0.014264762062945</v>
       </c>
       <c r="D82">
-        <v>9.688861707680337</v>
+        <v>2.956053995138761</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -29253,13 +29346,13 @@
         <v>348</v>
       </c>
       <c r="B83">
-        <v>-0.0044714872916435</v>
+        <v>-0.0014400052086357</v>
       </c>
       <c r="C83">
-        <v>-0.0013391082073518</v>
+        <v>-0.0003120407641864</v>
       </c>
       <c r="D83">
-        <v>0.0020423981040641</v>
+        <v>0.0014557148194222</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -29267,13 +29360,13 @@
         <v>349</v>
       </c>
       <c r="B84">
-        <v>-0.0525744392599648</v>
+        <v>-0.0092219525897758</v>
       </c>
       <c r="C84">
-        <v>-0.0171494684421075</v>
+        <v>-0.0030791050517514</v>
       </c>
       <c r="D84">
-        <v>0.0115342618518865</v>
+        <v>0.009660153300534199</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -29281,13 +29374,13 @@
         <v>350</v>
       </c>
       <c r="B85">
-        <v>-0.0112267643862325</v>
+        <v>-0.0070240337429207</v>
       </c>
       <c r="C85">
-        <v>-0.0029058602544759</v>
+        <v>-0.0006335487058153</v>
       </c>
       <c r="D85">
-        <v>0.0063076849028225</v>
+        <v>0.0073185486643817</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -29295,13 +29388,13 @@
         <v>351</v>
       </c>
       <c r="B86">
-        <v>-2.786265087219668</v>
+        <v>-4.604266585939934</v>
       </c>
       <c r="C86">
-        <v>2.1988457009937</v>
+        <v>-0.1610946600762464</v>
       </c>
       <c r="D86">
-        <v>8.214289453256146</v>
+        <v>2.271816136097634</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -29309,13 +29402,13 @@
         <v>352</v>
       </c>
       <c r="B87">
-        <v>-0.0040843661157776</v>
+        <v>-0.0013582608094532</v>
       </c>
       <c r="C87">
-        <v>-0.0012093996409148</v>
+        <v>-0.0003106496329419</v>
       </c>
       <c r="D87">
-        <v>0.001747550888315</v>
+        <v>0.0011871526573034</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -29323,13 +29416,13 @@
         <v>353</v>
       </c>
       <c r="B88">
-        <v>-0.0466403738741311</v>
+        <v>-0.0072524656414759</v>
       </c>
       <c r="C88">
-        <v>-0.0153621063357693</v>
+        <v>-0.0021052604074276</v>
       </c>
       <c r="D88">
-        <v>0.0102103460156978</v>
+        <v>0.00792063451792</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -29337,13 +29430,13 @@
         <v>354</v>
       </c>
       <c r="B89">
-        <v>-0.0104736177155591</v>
+        <v>-0.0073298904858175</v>
       </c>
       <c r="C89">
-        <v>-0.0026323891054475</v>
+        <v>-0.0007995906495706</v>
       </c>
       <c r="D89">
-        <v>0.0059824815935487</v>
+        <v>0.0062255751139378</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -29351,13 +29444,13 @@
         <v>355</v>
       </c>
       <c r="B90">
-        <v>-2.647342048379141</v>
+        <v>-3.788296911454047</v>
       </c>
       <c r="C90">
-        <v>1.91686539985017</v>
+        <v>-0.0270126939395381</v>
       </c>
       <c r="D90">
-        <v>7.050169402109522</v>
+        <v>2.64223513494995</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -29365,13 +29458,13 @@
         <v>356</v>
       </c>
       <c r="B91">
-        <v>-0.0036537792704286</v>
+        <v>-0.0010316856223021</v>
       </c>
       <c r="C91">
-        <v>-0.0010947960436669</v>
+        <v>-0.0002829312592958</v>
       </c>
       <c r="D91">
-        <v>0.0016373950926078</v>
+        <v>0.0010798060649894</v>
       </c>
     </row>
   </sheetData>

</xml_diff>